<commit_message>
correcgión de data 2026
</commit_message>
<xml_diff>
--- a/data/ep_mes_2026.xlsx
+++ b/data/ep_mes_2026.xlsx
@@ -5,12 +5,12 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\1. Proyectos\2. Data Richino\2026\enero - febrero\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\6. Código\10. st_seguimiento_unsch_2026\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FF7C70F7-E810-42D3-AB05-4AD09FDD963B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BE134798-2D60-4AC2-BF23-98077F07AB9B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-28920" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Hoja1" sheetId="1" r:id="rId1"/>
@@ -24795,11 +24795,11 @@
       <c r="B287">
         <v>60</v>
       </c>
-      <c r="C287" t="s">
+      <c r="C287">
+        <v>4</v>
+      </c>
+      <c r="D287" t="s">
         <v>660</v>
-      </c>
-      <c r="D287">
-        <v>0</v>
       </c>
       <c r="E287">
         <v>0</v>
@@ -24854,11 +24854,11 @@
       <c r="B288">
         <v>79</v>
       </c>
-      <c r="C288" t="s">
+      <c r="C288">
+        <v>4</v>
+      </c>
+      <c r="D288" t="s">
         <v>660</v>
-      </c>
-      <c r="D288">
-        <v>0</v>
       </c>
       <c r="E288">
         <v>0</v>
@@ -24913,11 +24913,11 @@
       <c r="B289">
         <v>143</v>
       </c>
-      <c r="C289" t="s">
+      <c r="C289">
+        <v>4</v>
+      </c>
+      <c r="D289" t="s">
         <v>660</v>
-      </c>
-      <c r="D289">
-        <v>0</v>
       </c>
       <c r="E289">
         <v>0</v>
@@ -24972,11 +24972,11 @@
       <c r="B290">
         <v>272</v>
       </c>
-      <c r="C290" t="s">
+      <c r="C290">
+        <v>4</v>
+      </c>
+      <c r="D290" t="s">
         <v>660</v>
-      </c>
-      <c r="D290">
-        <v>0</v>
       </c>
       <c r="E290">
         <v>0</v>
@@ -25031,11 +25031,11 @@
       <c r="B291">
         <v>267</v>
       </c>
-      <c r="C291" t="s">
+      <c r="C291">
+        <v>4</v>
+      </c>
+      <c r="D291" t="s">
         <v>660</v>
-      </c>
-      <c r="D291">
-        <v>0</v>
       </c>
       <c r="E291">
         <v>0</v>
@@ -25090,11 +25090,11 @@
       <c r="B292">
         <v>127</v>
       </c>
-      <c r="C292" t="s">
+      <c r="C292">
+        <v>4</v>
+      </c>
+      <c r="D292" t="s">
         <v>660</v>
-      </c>
-      <c r="D292">
-        <v>0</v>
       </c>
       <c r="E292">
         <v>0</v>
@@ -25149,11 +25149,11 @@
       <c r="B293">
         <v>429</v>
       </c>
-      <c r="C293" t="s">
+      <c r="C293">
+        <v>4</v>
+      </c>
+      <c r="D293" t="s">
         <v>660</v>
-      </c>
-      <c r="D293">
-        <v>0</v>
       </c>
       <c r="E293">
         <v>0</v>
@@ -25208,11 +25208,11 @@
       <c r="B294">
         <v>439</v>
       </c>
-      <c r="C294" t="s">
+      <c r="C294">
+        <v>4</v>
+      </c>
+      <c r="D294" t="s">
         <v>660</v>
-      </c>
-      <c r="D294">
-        <v>0</v>
       </c>
       <c r="E294">
         <v>0</v>
@@ -25267,11 +25267,11 @@
       <c r="B295">
         <v>106</v>
       </c>
-      <c r="C295" t="s">
+      <c r="C295">
+        <v>4</v>
+      </c>
+      <c r="D295" t="s">
         <v>660</v>
-      </c>
-      <c r="D295">
-        <v>0</v>
       </c>
       <c r="E295">
         <v>0</v>
@@ -25326,11 +25326,11 @@
       <c r="B296">
         <v>266</v>
       </c>
-      <c r="C296" t="s">
+      <c r="C296">
+        <v>4</v>
+      </c>
+      <c r="D296" t="s">
         <v>660</v>
-      </c>
-      <c r="D296">
-        <v>0</v>
       </c>
       <c r="E296">
         <v>0</v>
@@ -25385,11 +25385,11 @@
       <c r="B297">
         <v>106</v>
       </c>
-      <c r="C297" t="s">
+      <c r="C297">
+        <v>4</v>
+      </c>
+      <c r="D297" t="s">
         <v>660</v>
-      </c>
-      <c r="D297">
-        <v>0</v>
       </c>
       <c r="E297">
         <v>0</v>
@@ -25444,11 +25444,11 @@
       <c r="B298">
         <v>266</v>
       </c>
-      <c r="C298" t="s">
+      <c r="C298">
+        <v>4</v>
+      </c>
+      <c r="D298" t="s">
         <v>660</v>
-      </c>
-      <c r="D298">
-        <v>0</v>
       </c>
       <c r="E298">
         <v>0</v>

</xml_diff>